<commit_message>
Add month-end close: raw data generator, SQL ledger, checks and close report
</commit_message>
<xml_diff>
--- a/pack/DirectSportsGoods_FY26_management_pack.xlsx
+++ b/pack/DirectSportsGoods_FY26_management_pack.xlsx
@@ -39,7 +39,7 @@
     <numFmt numFmtId="170" formatCode="£#,##0"/>
     <numFmt numFmtId="171" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,6 +68,10 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="000000FF"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
     <font>
@@ -77,6 +81,13 @@
     <font>
       <b val="1"/>
       <i val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00008000"/>
+    </font>
+    <font>
+      <color rgb="000000FF"/>
     </font>
   </fonts>
   <fills count="5">
@@ -117,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -127,25 +138,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -154,17 +165,16 @@
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="171" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="11" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -727,7 +737,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="45" customHeight="1">
+    <row r="15" ht="30" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
           <t>What to do: review the peak trading plan before next November: stock depth on top sellers, site speed and checkout conversion, and whether extra search spend paid back. Set a spend cap per order for peak weeks.</t>
@@ -769,10 +779,10 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1">
+    <row r="23" ht="15" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Marketplace fees and marketing use placeholder assumptions with no citation yet. Those lines will move once benchmarks are sourced.</t>
+          <t>Marketing uses a placeholder assumption with no citation yet. That line will move once a benchmark is sourced.</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1338,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Marketplace fees *</t>
+          <t>Marketplace fees</t>
         </is>
       </c>
       <c r="B14" s="10">
@@ -2162,7 +2172,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Marketplace fees *</t>
+          <t>Marketplace fees</t>
         </is>
       </c>
       <c r="B13" s="10">
@@ -3265,7 +3275,7 @@
           <t>Opening cash</t>
         </is>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="30">
         <f>Assumptions!$B$21</f>
         <v/>
       </c>
@@ -3673,60 +3683,60 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="30" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Net cash flow</t>
         </is>
       </c>
-      <c r="B13" s="31">
+      <c r="B13" s="32">
         <f>B10+B11+B12</f>
         <v/>
       </c>
-      <c r="C13" s="31">
+      <c r="C13" s="32">
         <f>C10+C11+C12</f>
         <v/>
       </c>
-      <c r="D13" s="31">
+      <c r="D13" s="32">
         <f>D10+D11+D12</f>
         <v/>
       </c>
-      <c r="E13" s="31">
+      <c r="E13" s="32">
         <f>E10+E11+E12</f>
         <v/>
       </c>
-      <c r="F13" s="31">
+      <c r="F13" s="32">
         <f>F10+F11+F12</f>
         <v/>
       </c>
-      <c r="G13" s="31">
+      <c r="G13" s="32">
         <f>G10+G11+G12</f>
         <v/>
       </c>
-      <c r="H13" s="31">
+      <c r="H13" s="32">
         <f>H10+H11+H12</f>
         <v/>
       </c>
-      <c r="I13" s="31">
+      <c r="I13" s="32">
         <f>I10+I11+I12</f>
         <v/>
       </c>
-      <c r="J13" s="31">
+      <c r="J13" s="32">
         <f>J10+J11+J12</f>
         <v/>
       </c>
-      <c r="K13" s="31">
+      <c r="K13" s="32">
         <f>K10+K11+K12</f>
         <v/>
       </c>
-      <c r="L13" s="31">
+      <c r="L13" s="32">
         <f>L10+L11+L12</f>
         <v/>
       </c>
-      <c r="M13" s="31">
+      <c r="M13" s="32">
         <f>M10+M11+M12</f>
         <v/>
       </c>
-      <c r="N13" s="31">
+      <c r="N13" s="32">
         <f>SUM(B13:M13)</f>
         <v/>
       </c>
@@ -3826,7 +3836,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Blue = fictional company choice. Yellow = placeholder with no citation yet. Full sources in docs/assumptions.md.</t>
+          <t>Blue = hard-coded input. Yellow = placeholder with no citation yet. Full sources in docs/assumptions.md.</t>
         </is>
       </c>
     </row>
@@ -3848,7 +3858,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="32" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Budget net revenue, FY26</t>
         </is>
@@ -3856,14 +3866,14 @@
       <c r="B5" s="33" t="n">
         <v>48000000</v>
       </c>
-      <c r="C5" s="32" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Company assumption (fictional)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="32" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Website share of net revenue</t>
         </is>
@@ -3871,14 +3881,14 @@
       <c r="B6" s="34" t="n">
         <v>0.7</v>
       </c>
-      <c r="C6" s="32" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Company assumption (fictional)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="32" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Average order value, website (gross)</t>
         </is>
@@ -3886,14 +3896,14 @@
       <c r="B7" s="35" t="n">
         <v>62</v>
       </c>
-      <c r="C7" s="32" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Company assumption (fictional)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="32" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Average order value, marketplace (gross)</t>
         </is>
@@ -3901,7 +3911,7 @@
       <c r="B8" s="35" t="n">
         <v>45</v>
       </c>
-      <c r="C8" s="32" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Company assumption (fictional)</t>
         </is>
@@ -4003,7 +4013,7 @@
           <t>Delivery and fulfilment cost per order</t>
         </is>
       </c>
-      <c r="B15" s="28" t="n">
+      <c r="B15" s="35" t="n">
         <v>4.2</v>
       </c>
       <c r="C15" t="inlineStr">
@@ -4013,17 +4023,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="38" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Marketplace fees % of marketplace net revenue</t>
         </is>
       </c>
-      <c r="B16" s="39" t="n">
+      <c r="B16" s="36" t="n">
         <v>0.15</v>
       </c>
-      <c r="C16" s="38" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: no citation yet</t>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Amazon UK seller pricing, Sports and Outdoors referral fee (sell.amazon.co.uk/pricing, read 4 Oct 2026)</t>
         </is>
       </c>
     </row>
@@ -4043,7 +4053,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Other overheads per month</t>
         </is>
@@ -4051,14 +4061,14 @@
       <c r="B18" s="33" t="n">
         <v>300000</v>
       </c>
-      <c r="C18" s="32" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Company assumption (fictional)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="32" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Depreciation per month</t>
         </is>
@@ -4066,14 +4076,14 @@
       <c r="B19" s="33" t="n">
         <v>60000</v>
       </c>
-      <c r="C19" s="32" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Company assumption (fictional)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="32" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Capital expenditure per month</t>
         </is>
@@ -4081,14 +4091,14 @@
       <c r="B20" s="33" t="n">
         <v>70000</v>
       </c>
-      <c r="C20" s="32" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Company assumption (fictional)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Opening cash, 1 Feb 2025</t>
         </is>
@@ -4096,7 +4106,7 @@
       <c r="B21" s="33" t="n">
         <v>4000000</v>
       </c>
-      <c r="C21" s="32" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Company assumption (fictional)</t>
         </is>
@@ -4108,7 +4118,7 @@
           <t>Corporation tax main rate</t>
         </is>
       </c>
-      <c r="B22" s="40" t="n">
+      <c r="B22" s="34" t="n">
         <v>0.25</v>
       </c>
       <c r="C22" t="inlineStr">
@@ -4118,7 +4128,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="32" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Planned sales growth on FY25</t>
         </is>
@@ -4126,7 +4136,7 @@
       <c r="B23" s="34" t="n">
         <v>0.1</v>
       </c>
-      <c r="C23" s="32" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Company assumption (fictional)</t>
         </is>

</xml_diff>

<commit_message>
Fix corporation tax timing: quarterly instalments for profits above £1.5m
</commit_message>
<xml_diff>
--- a/pack/DirectSportsGoods_FY26_management_pack.xlsx
+++ b/pack/DirectSportsGoods_FY26_management_pack.xlsx
@@ -22548,7 +22548,7 @@
         </is>
       </c>
       <c r="F652" t="n">
-        <v>0</v>
+        <v>-131281.56</v>
       </c>
     </row>
     <row r="653">
@@ -22632,7 +22632,7 @@
         </is>
       </c>
       <c r="F655" t="n">
-        <v>0</v>
+        <v>-131281.56</v>
       </c>
     </row>
     <row r="656">
@@ -22716,7 +22716,7 @@
         </is>
       </c>
       <c r="F658" t="n">
-        <v>0</v>
+        <v>-147552.4</v>
       </c>
     </row>
     <row r="659">
@@ -22800,7 +22800,7 @@
         </is>
       </c>
       <c r="F661" t="n">
-        <v>-525126.24</v>
+        <v>-147552.4</v>
       </c>
     </row>
     <row r="662">

</xml_diff>

<commit_message>
Cite marketing spend from ASOS FY25 and rebuild all stages
</commit_message>
<xml_diff>
--- a/pack/DirectSportsGoods_FY26_management_pack.xlsx
+++ b/pack/DirectSportsGoods_FY26_management_pack.xlsx
@@ -90,7 +90,7 @@
       <color rgb="000000FF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -105,11 +105,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -128,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -173,8 +168,6 @@
     <xf numFmtId="169" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="171" fontId="11" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -639,7 +632,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Benchmarks are calibrated on Frasers Group plc's published accounts. Lines marked * use placeholder assumptions.</t>
+          <t>Benchmarks come from the published accounts of Frasers Group, Debenhams Group and ASOS, and Amazon UK's seller fees.</t>
         </is>
       </c>
     </row>
@@ -654,7 +647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -684,7 +677,7 @@
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Net revenue was £49.15m, £1,147k (+2.4%) ahead of budget. Operating profit was £2.36m, £517k (-18.0%) behind. Sales grew in the channel that earns least, and costs per order rose. Gross margin finished at 50.7% against 51.1% budgeted, mostly from January clearance discounting (about £177k).</t>
+          <t>Net revenue was £49.15m, £1,147k (+2.4%) ahead of budget. Operating profit was £3.46m, £496k (-12.5%) behind. Sales grew in the channel that earns least, and costs per order rose. Gross margin finished at 50.7% against 51.1% budgeted, mostly from January clearance discounting (about £177k).</t>
         </is>
       </c>
     </row>
@@ -705,7 +698,7 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Why it matters: every £1 of marketplace sales earned 22% contribution against 30% on the website, because of marketplace fees. The extra sales added £318k of contribution.</t>
+          <t>Why it matters: every £1 of marketplace sales earned 22% contribution against 33% on the website, because of marketplace fees. The extra sales added £318k of contribution.</t>
         </is>
       </c>
     </row>
@@ -726,14 +719,14 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>What happened: £619k of the shortfall was in November and December. Black Friday and Christmas orders came in below plan, even after an extra £93k of paid search in November.</t>
+          <t>What happened: £619k of the shortfall was in November and December. Black Friday and Christmas orders came in below plan, even after an extra £63k of paid search in November.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Why it matters: this is the higher-margin channel. Website contribution was £779k behind budget, more than the whole profit gap. The marketplace beat only partly offset it.</t>
+          <t>Why it matters: this is the higher-margin channel. Website contribution was £758k behind budget, more than the whole profit gap. The marketplace beat only partly offset it.</t>
         </is>
       </c>
     </row>
@@ -769,20 +762,6 @@
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t>What to do: retender the carrier contract, test a higher free-delivery threshold, and pass part of the increase on in the delivery charge. Put the new rate in next year's budget.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Caveat</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>Marketing uses a placeholder assumption with no citation yet. That line will move once a benchmark is sourced.</t>
         </is>
       </c>
     </row>
@@ -797,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1397,7 +1376,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Marketing *</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="B15" s="10">
@@ -1927,13 +1906,6 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>* Uses a placeholder assumption with no citation yet. See the Assumptions sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Payroll, overheads and depreciation are central costs, so they only appear in the Total view.</t>
         </is>
@@ -1958,7 +1930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2195,7 +2167,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Marketing *</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="B14" s="10">
@@ -2391,52 +2363,68 @@
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>* Uses a placeholder assumption with no citation yet. See the Assumptions sheet.</t>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>By channel</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Variance £</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>Variance %</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>By channel</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>Actual</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>Budget</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>Variance £</t>
-        </is>
-      </c>
-      <c r="E26" s="9" t="inlineStr">
-        <is>
-          <t>Variance %</t>
-        </is>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Website net revenue</t>
+        </is>
+      </c>
+      <c r="B26" s="10">
+        <f>SUM(SUMIFS(d_val,d_scn,"Actual",d_ch,"Website",d_line,{"Gross sales","Returns"}))</f>
+        <v/>
+      </c>
+      <c r="C26" s="10">
+        <f>SUM(SUMIFS(d_val,d_scn,"Budget",d_ch,"Website",d_line,{"Gross sales","Returns"}))</f>
+        <v/>
+      </c>
+      <c r="D26" s="22">
+        <f>B26-C26</f>
+        <v/>
+      </c>
+      <c r="E26" s="23">
+        <f>IF(C26=0,"",D26/ABS(C26))</f>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Website net revenue</t>
+          <t>Website contribution</t>
         </is>
       </c>
       <c r="B27" s="10">
-        <f>SUM(SUMIFS(d_val,d_scn,"Actual",d_ch,"Website",d_line,{"Gross sales","Returns"}))</f>
+        <f>SUM(SUMIFS(d_val,d_scn,"Actual",d_ch,"Website",d_line,{"Gross sales","Returns","Cost of goods sold","Delivery","Marketplace fees","Marketing"}))</f>
         <v/>
       </c>
       <c r="C27" s="10">
-        <f>SUM(SUMIFS(d_val,d_scn,"Budget",d_ch,"Website",d_line,{"Gross sales","Returns"}))</f>
+        <f>SUM(SUMIFS(d_val,d_scn,"Budget",d_ch,"Website",d_line,{"Gross sales","Returns","Cost of goods sold","Delivery","Marketplace fees","Marketing"}))</f>
         <v/>
       </c>
       <c r="D27" s="22">
@@ -2451,15 +2439,15 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Website contribution</t>
+          <t>Marketplace net revenue</t>
         </is>
       </c>
       <c r="B28" s="10">
-        <f>SUM(SUMIFS(d_val,d_scn,"Actual",d_ch,"Website",d_line,{"Gross sales","Returns","Cost of goods sold","Delivery","Marketplace fees","Marketing"}))</f>
+        <f>SUM(SUMIFS(d_val,d_scn,"Actual",d_ch,"Marketplace",d_line,{"Gross sales","Returns"}))</f>
         <v/>
       </c>
       <c r="C28" s="10">
-        <f>SUM(SUMIFS(d_val,d_scn,"Budget",d_ch,"Website",d_line,{"Gross sales","Returns","Cost of goods sold","Delivery","Marketplace fees","Marketing"}))</f>
+        <f>SUM(SUMIFS(d_val,d_scn,"Budget",d_ch,"Marketplace",d_line,{"Gross sales","Returns"}))</f>
         <v/>
       </c>
       <c r="D28" s="22">
@@ -2474,15 +2462,15 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Marketplace net revenue</t>
+          <t>Marketplace contribution</t>
         </is>
       </c>
       <c r="B29" s="10">
-        <f>SUM(SUMIFS(d_val,d_scn,"Actual",d_ch,"Marketplace",d_line,{"Gross sales","Returns"}))</f>
+        <f>SUM(SUMIFS(d_val,d_scn,"Actual",d_ch,"Marketplace",d_line,{"Gross sales","Returns","Cost of goods sold","Delivery","Marketplace fees","Marketing"}))</f>
         <v/>
       </c>
       <c r="C29" s="10">
-        <f>SUM(SUMIFS(d_val,d_scn,"Budget",d_ch,"Marketplace",d_line,{"Gross sales","Returns"}))</f>
+        <f>SUM(SUMIFS(d_val,d_scn,"Budget",d_ch,"Marketplace",d_line,{"Gross sales","Returns","Cost of goods sold","Delivery","Marketplace fees","Marketing"}))</f>
         <v/>
       </c>
       <c r="D29" s="22">
@@ -2491,29 +2479,6 @@
       </c>
       <c r="E29" s="23">
         <f>IF(C29=0,"",D29/ABS(C29))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Marketplace contribution</t>
-        </is>
-      </c>
-      <c r="B30" s="10">
-        <f>SUM(SUMIFS(d_val,d_scn,"Actual",d_ch,"Marketplace",d_line,{"Gross sales","Returns","Cost of goods sold","Delivery","Marketplace fees","Marketing"}))</f>
-        <v/>
-      </c>
-      <c r="C30" s="10">
-        <f>SUM(SUMIFS(d_val,d_scn,"Budget",d_ch,"Marketplace",d_line,{"Gross sales","Returns","Cost of goods sold","Delivery","Marketplace fees","Marketing"}))</f>
-        <v/>
-      </c>
-      <c r="D30" s="22">
-        <f>B30-C30</f>
-        <v/>
-      </c>
-      <c r="E30" s="23">
-        <f>IF(C30=0,"",D30/ABS(C30))</f>
         <v/>
       </c>
     </row>
@@ -2528,7 +2493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3141,13 +3106,6 @@
       <c r="O13" s="24">
         <f>-SUMIFS(d_val,d_scn,"Budget",d_ch,"*",d_line,"Returns",d_per,"&gt;=1")/SUMIFS(d_val,d_scn,"Budget",d_ch,"*",d_line,"Gross sales",d_per,"&gt;=1")</f>
         <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>* Uses a placeholder assumption with no citation yet. See the Assumptions sheet.</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -3836,7 +3794,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Blue = hard-coded input. Yellow = placeholder with no citation yet. Full sources in docs/assumptions.md.</t>
+          <t>Blue = hard-coded input. Full sources in docs/assumptions.md.</t>
         </is>
       </c>
     </row>
@@ -4038,17 +3996,17 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="38" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Marketing budget % of website net revenue</t>
         </is>
       </c>
-      <c r="B17" s="39" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C17" s="38" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: no citation yet</t>
+      <c r="B17" s="36" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ASOS AR 2025, p.49 (6.8% of revenue; ASOS sells through its own site)</t>
         </is>
       </c>
     </row>
@@ -6364,7 +6322,7 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>-189073.4</v>
+        <v>-128569.91</v>
       </c>
     </row>
     <row r="75">
@@ -6392,7 +6350,7 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>-220585.63</v>
+        <v>-149998.23</v>
       </c>
     </row>
     <row r="76">
@@ -6420,7 +6378,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>-220585.63</v>
+        <v>-149998.23</v>
       </c>
     </row>
     <row r="77">
@@ -6448,7 +6406,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>-268626.8</v>
+        <v>-182666.23</v>
       </c>
     </row>
     <row r="78">
@@ -6476,7 +6434,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>-286535.26</v>
+        <v>-194843.98</v>
       </c>
     </row>
     <row r="79">
@@ -6504,7 +6462,7 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>-304443.71</v>
+        <v>-207021.72</v>
       </c>
     </row>
     <row r="80">
@@ -6532,7 +6490,7 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>-322352.16</v>
+        <v>-219199.47</v>
       </c>
     </row>
     <row r="81">
@@ -6560,7 +6518,7 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>-286535.26</v>
+        <v>-194843.98</v>
       </c>
     </row>
     <row r="82">
@@ -6588,7 +6546,7 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>-268626.8</v>
+        <v>-182666.23</v>
       </c>
     </row>
     <row r="83">
@@ -6616,7 +6574,7 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>-346634.56</v>
+        <v>-235711.5</v>
       </c>
     </row>
     <row r="84">
@@ -6644,7 +6602,7 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>-362390.68</v>
+        <v>-246425.66</v>
       </c>
     </row>
     <row r="85">
@@ -6672,7 +6630,7 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>-283610.1</v>
+        <v>-192854.87</v>
       </c>
     </row>
     <row r="86">
@@ -12076,7 +12034,7 @@
         </is>
       </c>
       <c r="F278" t="n">
-        <v>-191497.25</v>
+        <v>-130218.13</v>
       </c>
     </row>
     <row r="279">
@@ -12104,7 +12062,7 @@
         </is>
       </c>
       <c r="F279" t="n">
-        <v>-209356.13</v>
+        <v>-142362.17</v>
       </c>
     </row>
     <row r="280">
@@ -12132,7 +12090,7 @@
         </is>
       </c>
       <c r="F280" t="n">
-        <v>-228400.05</v>
+        <v>-155312.03</v>
       </c>
     </row>
     <row r="281">
@@ -12160,7 +12118,7 @@
         </is>
       </c>
       <c r="F281" t="n">
-        <v>-274570.48</v>
+        <v>-186707.92</v>
       </c>
     </row>
     <row r="282">
@@ -12188,7 +12146,7 @@
         </is>
       </c>
       <c r="F282" t="n">
-        <v>-286243.19</v>
+        <v>-194645.37</v>
       </c>
     </row>
     <row r="283">
@@ -12216,7 +12174,7 @@
         </is>
       </c>
       <c r="F283" t="n">
-        <v>-294460.56</v>
+        <v>-200233.18</v>
       </c>
     </row>
     <row r="284">
@@ -12244,7 +12202,7 @@
         </is>
       </c>
       <c r="F284" t="n">
-        <v>-326932.18</v>
+        <v>-222313.88</v>
       </c>
     </row>
     <row r="285">
@@ -12272,7 +12230,7 @@
         </is>
       </c>
       <c r="F285" t="n">
-        <v>-274895.91</v>
+        <v>-186929.22</v>
       </c>
     </row>
     <row r="286">
@@ -12300,7 +12258,7 @@
         </is>
       </c>
       <c r="F286" t="n">
-        <v>-264511.41</v>
+        <v>-179867.76</v>
       </c>
     </row>
     <row r="287">
@@ -12328,7 +12286,7 @@
         </is>
       </c>
       <c r="F287" t="n">
-        <v>-439431.7</v>
+        <v>-298813.55</v>
       </c>
     </row>
     <row r="288">
@@ -12356,7 +12314,7 @@
         </is>
       </c>
       <c r="F288" t="n">
-        <v>-363269.86</v>
+        <v>-247023.5</v>
       </c>
     </row>
     <row r="289">
@@ -12384,7 +12342,7 @@
         </is>
       </c>
       <c r="F289" t="n">
-        <v>-272835.72</v>
+        <v>-185528.29</v>
       </c>
     </row>
     <row r="290">
@@ -17788,7 +17746,7 @@
         </is>
       </c>
       <c r="F482" t="n">
-        <v>-170121.79</v>
+        <v>-115682.82</v>
       </c>
     </row>
     <row r="483">
@@ -17816,7 +17774,7 @@
         </is>
       </c>
       <c r="F483" t="n">
-        <v>-197340.93</v>
+        <v>-134191.84</v>
       </c>
     </row>
     <row r="484">
@@ -17844,7 +17802,7 @@
         </is>
       </c>
       <c r="F484" t="n">
-        <v>-198335.28</v>
+        <v>-134867.99</v>
       </c>
     </row>
     <row r="485">
@@ -17872,7 +17830,7 @@
         </is>
       </c>
       <c r="F485" t="n">
-        <v>-256156.26</v>
+        <v>-174186.26</v>
       </c>
     </row>
     <row r="486">
@@ -17900,7 +17858,7 @@
         </is>
       </c>
       <c r="F486" t="n">
-        <v>-267240.34</v>
+        <v>-181723.43</v>
       </c>
     </row>
     <row r="487">
@@ -17928,7 +17886,7 @@
         </is>
       </c>
       <c r="F487" t="n">
-        <v>-278252.97</v>
+        <v>-189212.02</v>
       </c>
     </row>
     <row r="488">
@@ -17956,7 +17914,7 @@
         </is>
       </c>
       <c r="F488" t="n">
-        <v>-277439.18</v>
+        <v>-188658.65</v>
       </c>
     </row>
     <row r="489">
@@ -17984,7 +17942,7 @@
         </is>
       </c>
       <c r="F489" t="n">
-        <v>-267953.92</v>
+        <v>-182208.66</v>
       </c>
     </row>
     <row r="490">
@@ -18012,7 +17970,7 @@
         </is>
       </c>
       <c r="F490" t="n">
-        <v>-252050.12</v>
+        <v>-171394.08</v>
       </c>
     </row>
     <row r="491">
@@ -18040,7 +17998,7 @@
         </is>
       </c>
       <c r="F491" t="n">
-        <v>-310915.21</v>
+        <v>-211422.34</v>
       </c>
     </row>
     <row r="492">
@@ -18068,7 +18026,7 @@
         </is>
       </c>
       <c r="F492" t="n">
-        <v>-334048.75</v>
+        <v>-227153.15</v>
       </c>
     </row>
     <row r="493">
@@ -18096,7 +18054,7 @@
         </is>
       </c>
       <c r="F493" t="n">
-        <v>-252947.09</v>
+        <v>-172004.02</v>
       </c>
     </row>
     <row r="494">
@@ -22548,7 +22506,7 @@
         </is>
       </c>
       <c r="F652" t="n">
-        <v>-131281.56</v>
+        <v>-192537.6</v>
       </c>
     </row>
     <row r="653">
@@ -22632,7 +22590,7 @@
         </is>
       </c>
       <c r="F655" t="n">
-        <v>-131281.56</v>
+        <v>-192537.6</v>
       </c>
     </row>
     <row r="656">
@@ -22716,7 +22674,7 @@
         </is>
       </c>
       <c r="F658" t="n">
-        <v>-147552.4</v>
+        <v>-216080.48</v>
       </c>
     </row>
     <row r="659">
@@ -22800,7 +22758,7 @@
         </is>
       </c>
       <c r="F661" t="n">
-        <v>-147552.4</v>
+        <v>-216080.48</v>
       </c>
     </row>
     <row r="662">

</xml_diff>